<commit_message>
move location of summaries up one level, look at the code for sup table 5
</commit_message>
<xml_diff>
--- a/output_for_paper/sup_table_s5_syn_SBS_skin_missed_sig.xlsx
+++ b/output_for_paper/sup_table_s5_syn_SBS_skin_missed_sig.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -372,27 +372,122 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>sigpro</t>
+          <t>musical</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>fitms</t>
+          <t>fitms_0.010</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>fitms_0.030</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.050</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.060</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.200</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.005</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.001</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>fitms_0.100</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mp</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>yapsa_0.03</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>deconstruct_0.03</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>yapsa_0.01</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>deconstruct_0.06</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>yapsa_0.06</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>mutsig</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>yapsa_0.00</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>deconstruct_0.10</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>deconstruct_0.00</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>yapsa_0.10</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>QP_null</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>sigest</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>msa</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>msa_opt</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>mp</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>msa</t>
         </is>
       </c>
     </row>
@@ -403,25 +498,82 @@
         </is>
       </c>
       <c r="B2">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C2">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E2">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="F2">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="G2">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="H2">
-        <v>42</v>
+        <v>56</v>
+      </c>
+      <c r="I2">
+        <v>56</v>
+      </c>
+      <c r="J2">
+        <v>56</v>
+      </c>
+      <c r="K2">
+        <v>56</v>
+      </c>
+      <c r="L2">
+        <v>56</v>
+      </c>
+      <c r="M2">
+        <v>56</v>
+      </c>
+      <c r="N2">
+        <v>54</v>
+      </c>
+      <c r="O2">
+        <v>55</v>
+      </c>
+      <c r="P2">
+        <v>33</v>
+      </c>
+      <c r="Q2">
+        <v>56</v>
+      </c>
+      <c r="R2">
+        <v>56</v>
+      </c>
+      <c r="S2">
+        <v>15</v>
+      </c>
+      <c r="T2">
+        <v>15</v>
+      </c>
+      <c r="U2">
+        <v>57</v>
+      </c>
+      <c r="V2">
+        <v>55</v>
+      </c>
+      <c r="W2">
+        <v>56</v>
+      </c>
+      <c r="X2">
+        <v>11</v>
+      </c>
+      <c r="Y2">
+        <v>11</v>
+      </c>
+      <c r="Z2">
+        <v>38</v>
+      </c>
+      <c r="AA2">
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -431,25 +583,82 @@
         </is>
       </c>
       <c r="B3">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H3">
+        <v>9</v>
+      </c>
+      <c r="I3">
+        <v>9</v>
+      </c>
+      <c r="J3">
+        <v>9</v>
+      </c>
+      <c r="K3">
+        <v>9</v>
+      </c>
+      <c r="L3">
+        <v>9</v>
+      </c>
+      <c r="M3">
         <v>8</v>
+      </c>
+      <c r="N3">
+        <v>7</v>
+      </c>
+      <c r="O3">
+        <v>7</v>
+      </c>
+      <c r="P3">
+        <v>7</v>
+      </c>
+      <c r="Q3">
+        <v>9</v>
+      </c>
+      <c r="R3">
+        <v>9</v>
+      </c>
+      <c r="S3">
+        <v>7</v>
+      </c>
+      <c r="T3">
+        <v>7</v>
+      </c>
+      <c r="U3">
+        <v>9</v>
+      </c>
+      <c r="V3">
+        <v>7</v>
+      </c>
+      <c r="W3">
+        <v>9</v>
+      </c>
+      <c r="X3">
+        <v>4</v>
+      </c>
+      <c r="Y3">
+        <v>4</v>
+      </c>
+      <c r="Z3">
+        <v>8</v>
+      </c>
+      <c r="AA3">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -459,25 +668,82 @@
         </is>
       </c>
       <c r="B4">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D4">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="E4">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F4">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="G4">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="H4">
+        <v>38</v>
+      </c>
+      <c r="I4">
+        <v>38</v>
+      </c>
+      <c r="J4">
+        <v>37</v>
+      </c>
+      <c r="K4">
+        <v>37</v>
+      </c>
+      <c r="L4">
+        <v>38</v>
+      </c>
+      <c r="M4">
+        <v>61</v>
+      </c>
+      <c r="N4">
+        <v>28</v>
+      </c>
+      <c r="O4">
+        <v>35</v>
+      </c>
+      <c r="P4">
+        <v>26</v>
+      </c>
+      <c r="Q4">
         <v>42</v>
+      </c>
+      <c r="R4">
+        <v>46</v>
+      </c>
+      <c r="S4">
+        <v>24</v>
+      </c>
+      <c r="T4">
+        <v>24</v>
+      </c>
+      <c r="U4">
+        <v>52</v>
+      </c>
+      <c r="V4">
+        <v>26</v>
+      </c>
+      <c r="W4">
+        <v>58</v>
+      </c>
+      <c r="X4">
+        <v>13</v>
+      </c>
+      <c r="Y4">
+        <v>13</v>
+      </c>
+      <c r="Z4">
+        <v>41</v>
+      </c>
+      <c r="AA4">
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -487,25 +753,82 @@
         </is>
       </c>
       <c r="B5">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
         <v>6</v>
       </c>
-      <c r="D5">
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>7</v>
+      </c>
+      <c r="N5">
+        <v>4</v>
+      </c>
+      <c r="O5">
         <v>5</v>
       </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>7</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>5</v>
+      <c r="P5">
+        <v>4</v>
+      </c>
+      <c r="Q5">
+        <v>8</v>
+      </c>
+      <c r="R5">
+        <v>8</v>
+      </c>
+      <c r="S5">
+        <v>4</v>
+      </c>
+      <c r="T5">
+        <v>4</v>
+      </c>
+      <c r="U5">
+        <v>9</v>
+      </c>
+      <c r="V5">
+        <v>4</v>
+      </c>
+      <c r="W5">
+        <v>9</v>
+      </c>
+      <c r="X5">
+        <v>3</v>
+      </c>
+      <c r="Y5">
+        <v>3</v>
+      </c>
+      <c r="Z5">
+        <v>13</v>
+      </c>
+      <c r="AA5">
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -515,25 +838,82 @@
         </is>
       </c>
       <c r="B6">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C6">
+        <v>25</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>9</v>
+      </c>
+      <c r="I6">
+        <v>11</v>
+      </c>
+      <c r="J6">
+        <v>9</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
         <v>22</v>
       </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6">
+      <c r="N6">
+        <v>10</v>
+      </c>
+      <c r="O6">
+        <v>10</v>
+      </c>
+      <c r="P6">
+        <v>7</v>
+      </c>
+      <c r="Q6">
+        <v>13</v>
+      </c>
+      <c r="R6">
+        <v>14</v>
+      </c>
+      <c r="S6">
+        <v>6</v>
+      </c>
+      <c r="T6">
+        <v>6</v>
+      </c>
+      <c r="U6">
+        <v>18</v>
+      </c>
+      <c r="V6">
+        <v>7</v>
+      </c>
+      <c r="W6">
+        <v>18</v>
+      </c>
+      <c r="X6">
+        <v>1</v>
+      </c>
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6">
         <v>8</v>
       </c>
-      <c r="F6">
-        <v>15</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
+      <c r="AA6">
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -543,25 +923,82 @@
         </is>
       </c>
       <c r="B7">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C7">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F7">
+        <v>38</v>
+      </c>
+      <c r="G7">
+        <v>38</v>
+      </c>
+      <c r="H7">
+        <v>38</v>
+      </c>
+      <c r="I7">
+        <v>38</v>
+      </c>
+      <c r="J7">
+        <v>39</v>
+      </c>
+      <c r="K7">
+        <v>39</v>
+      </c>
+      <c r="L7">
+        <v>38</v>
+      </c>
+      <c r="M7">
+        <v>49</v>
+      </c>
+      <c r="N7">
+        <v>27</v>
+      </c>
+      <c r="O7">
+        <v>32</v>
+      </c>
+      <c r="P7">
+        <v>11</v>
+      </c>
+      <c r="Q7">
+        <v>45</v>
+      </c>
+      <c r="R7">
+        <v>42</v>
+      </c>
+      <c r="S7">
+        <v>4</v>
+      </c>
+      <c r="T7">
+        <v>4</v>
+      </c>
+      <c r="U7">
+        <v>56</v>
+      </c>
+      <c r="V7">
+        <v>26</v>
+      </c>
+      <c r="W7">
         <v>55</v>
       </c>
-      <c r="G7">
-        <v>57</v>
-      </c>
-      <c r="H7">
-        <v>20</v>
+      <c r="X7">
+        <v>5</v>
+      </c>
+      <c r="Y7">
+        <v>5</v>
+      </c>
+      <c r="Z7">
+        <v>33</v>
+      </c>
+      <c r="AA7">
+        <v>65</v>
       </c>
     </row>
     <row r="8">
@@ -571,25 +1008,82 @@
         </is>
       </c>
       <c r="B8">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C8">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D8">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F8">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G8">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H8">
-        <v>16</v>
+        <v>45</v>
+      </c>
+      <c r="I8">
+        <v>45</v>
+      </c>
+      <c r="J8">
+        <v>45</v>
+      </c>
+      <c r="K8">
+        <v>45</v>
+      </c>
+      <c r="L8">
+        <v>45</v>
+      </c>
+      <c r="M8">
+        <v>60</v>
+      </c>
+      <c r="N8">
+        <v>40</v>
+      </c>
+      <c r="O8">
+        <v>42</v>
+      </c>
+      <c r="P8">
+        <v>21</v>
+      </c>
+      <c r="Q8">
+        <v>59</v>
+      </c>
+      <c r="R8">
+        <v>54</v>
+      </c>
+      <c r="S8">
+        <v>14</v>
+      </c>
+      <c r="T8">
+        <v>14</v>
+      </c>
+      <c r="U8">
+        <v>65</v>
+      </c>
+      <c r="V8">
+        <v>36</v>
+      </c>
+      <c r="W8">
+        <v>65</v>
+      </c>
+      <c r="X8">
+        <v>10</v>
+      </c>
+      <c r="Y8">
+        <v>10</v>
+      </c>
+      <c r="Z8">
+        <v>29</v>
+      </c>
+      <c r="AA8">
+        <v>60</v>
       </c>
     </row>
     <row r="9">
@@ -599,13 +1093,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>10</v>
       </c>
       <c r="D9">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>15</v>
@@ -614,94 +1108,152 @@
         <v>15</v>
       </c>
       <c r="G9">
+        <v>15</v>
+      </c>
+      <c r="H9">
+        <v>15</v>
+      </c>
+      <c r="I9">
+        <v>15</v>
+      </c>
+      <c r="J9">
+        <v>15</v>
+      </c>
+      <c r="K9">
+        <v>15</v>
+      </c>
+      <c r="L9">
+        <v>15</v>
+      </c>
+      <c r="M9">
+        <v>15</v>
+      </c>
+      <c r="N9">
+        <v>15</v>
+      </c>
+      <c r="O9">
+        <v>15</v>
+      </c>
+      <c r="P9">
+        <v>12</v>
+      </c>
+      <c r="Q9">
+        <v>15</v>
+      </c>
+      <c r="R9">
+        <v>15</v>
+      </c>
+      <c r="S9">
+        <v>2</v>
+      </c>
+      <c r="T9">
+        <v>2</v>
+      </c>
+      <c r="U9">
+        <v>17</v>
+      </c>
+      <c r="V9">
         <v>14</v>
       </c>
-      <c r="H9">
-        <v>9</v>
+      <c r="W9">
+        <v>17</v>
+      </c>
+      <c r="X9">
+        <v>4</v>
+      </c>
+      <c r="Y9">
+        <v>4</v>
+      </c>
+      <c r="Z9">
+        <v>16</v>
+      </c>
+      <c r="AA9">
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SBS17a</t>
+          <t>SBS40</t>
         </is>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SBS38</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>15</v>
-      </c>
-      <c r="C11">
-        <v>7</v>
-      </c>
-      <c r="D11">
-        <v>15</v>
-      </c>
-      <c r="E11">
-        <v>15</v>
-      </c>
-      <c r="F11">
-        <v>15</v>
-      </c>
-      <c r="G11">
-        <v>14</v>
-      </c>
-      <c r="H11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SBS40</t>
-        </is>
-      </c>
-      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>10</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10">
+        <v>18</v>
+      </c>
+      <c r="N10">
+        <v>15</v>
+      </c>
+      <c r="O10">
+        <v>13</v>
+      </c>
+      <c r="P10">
+        <v>11</v>
+      </c>
+      <c r="Q10">
+        <v>17</v>
+      </c>
+      <c r="R10">
+        <v>18</v>
+      </c>
+      <c r="S10">
+        <v>11</v>
+      </c>
+      <c r="T10">
+        <v>11</v>
+      </c>
+      <c r="U10">
+        <v>17</v>
+      </c>
+      <c r="V10">
+        <v>11</v>
+      </c>
+      <c r="W10">
+        <v>22</v>
+      </c>
+      <c r="X10">
+        <v>8</v>
+      </c>
+      <c r="Y10">
+        <v>8</v>
+      </c>
+      <c r="Z10">
         <v>21</v>
       </c>
-      <c r="C12">
-        <v>7</v>
-      </c>
-      <c r="D12">
-        <v>18</v>
-      </c>
-      <c r="E12">
-        <v>9</v>
-      </c>
-      <c r="F12">
-        <v>17</v>
-      </c>
-      <c r="G12">
-        <v>14</v>
-      </c>
-      <c r="H12">
-        <v>12</v>
+      <c r="AA10">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
regenerate outputs; delete old outputs
</commit_message>
<xml_diff>
--- a/output_for_paper/sup_table_s5_syn_SBS_skin_missed_sig.xlsx
+++ b/output_for_paper/sup_table_s5_syn_SBS_skin_missed_sig.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -417,77 +417,82 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>sigpro</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>mp</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>yapsa_0.03</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>deconstruct_0.03</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>yapsa_0.01</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>deconstruct_0.06</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>yapsa_0.06</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>mutsig</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>yapsa_0.00</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>deconstruct_0.10</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>deconstruct_0.00</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>yapsa_0.10</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>QP_null</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>sigest</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>msa</t>
-        </is>
-      </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>msa_opt</t>
+          <t>siglasso</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>siglasso_wprior</t>
         </is>
       </c>
     </row>
@@ -531,48 +536,51 @@
         <v>56</v>
       </c>
       <c r="M2">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="N2">
+        <v>56</v>
+      </c>
+      <c r="O2">
         <v>54</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>55</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>33</v>
       </c>
-      <c r="Q2">
-        <v>56</v>
-      </c>
       <c r="R2">
         <v>56</v>
       </c>
       <c r="S2">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="T2">
         <v>15</v>
       </c>
       <c r="U2">
+        <v>15</v>
+      </c>
+      <c r="V2">
         <v>57</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>55</v>
       </c>
-      <c r="W2">
-        <v>56</v>
-      </c>
       <c r="X2">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="Y2">
         <v>11</v>
       </c>
       <c r="Z2">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="AA2">
+        <v>56</v>
+      </c>
+      <c r="AB2">
         <v>56</v>
       </c>
     </row>
@@ -619,7 +627,7 @@
         <v>8</v>
       </c>
       <c r="N3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O3">
         <v>7</v>
@@ -628,36 +636,39 @@
         <v>7</v>
       </c>
       <c r="Q3">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R3">
         <v>9</v>
       </c>
       <c r="S3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T3">
         <v>7</v>
       </c>
       <c r="U3">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V3">
+        <v>9</v>
+      </c>
+      <c r="W3">
         <v>7</v>
       </c>
-      <c r="W3">
-        <v>9</v>
-      </c>
       <c r="X3">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="Y3">
         <v>4</v>
       </c>
       <c r="Z3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AA3">
+        <v>10</v>
+      </c>
+      <c r="AB3">
         <v>10</v>
       </c>
     </row>
@@ -701,49 +712,52 @@
         <v>38</v>
       </c>
       <c r="M4">
+        <v>46</v>
+      </c>
+      <c r="N4">
         <v>61</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>28</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>35</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>26</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>42</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>46</v>
-      </c>
-      <c r="S4">
-        <v>24</v>
       </c>
       <c r="T4">
         <v>24</v>
       </c>
       <c r="U4">
+        <v>24</v>
+      </c>
+      <c r="V4">
         <v>52</v>
       </c>
-      <c r="V4">
+      <c r="W4">
         <v>26</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <v>58</v>
-      </c>
-      <c r="X4">
-        <v>13</v>
       </c>
       <c r="Y4">
         <v>13</v>
       </c>
       <c r="Z4">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="AA4">
-        <v>67</v>
+        <v>66</v>
+      </c>
+      <c r="AB4">
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -789,46 +803,49 @@
         <v>7</v>
       </c>
       <c r="N5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O5">
+        <v>4</v>
+      </c>
+      <c r="P5">
         <v>5</v>
       </c>
-      <c r="P5">
-        <v>4</v>
-      </c>
       <c r="Q5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="R5">
         <v>8</v>
       </c>
       <c r="S5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="T5">
         <v>4</v>
       </c>
       <c r="U5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="V5">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="W5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="X5">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="Y5">
         <v>3</v>
       </c>
       <c r="Z5">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="AA5">
-        <v>23</v>
+        <v>15</v>
+      </c>
+      <c r="AB5">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -871,49 +888,52 @@
         <v>9</v>
       </c>
       <c r="M6">
+        <v>20</v>
+      </c>
+      <c r="N6">
         <v>22</v>
       </c>
-      <c r="N6">
-        <v>10</v>
-      </c>
       <c r="O6">
         <v>10</v>
       </c>
       <c r="P6">
+        <v>10</v>
+      </c>
+      <c r="Q6">
         <v>7</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>13</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>14</v>
-      </c>
-      <c r="S6">
-        <v>6</v>
       </c>
       <c r="T6">
         <v>6</v>
       </c>
       <c r="U6">
+        <v>6</v>
+      </c>
+      <c r="V6">
         <v>18</v>
       </c>
-      <c r="V6">
+      <c r="W6">
         <v>7</v>
       </c>
-      <c r="W6">
+      <c r="X6">
         <v>18</v>
-      </c>
-      <c r="X6">
-        <v>1</v>
       </c>
       <c r="Y6">
         <v>1</v>
       </c>
       <c r="Z6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA6">
-        <v>23</v>
+        <v>42</v>
+      </c>
+      <c r="AB6">
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -956,49 +976,52 @@
         <v>38</v>
       </c>
       <c r="M7">
+        <v>41</v>
+      </c>
+      <c r="N7">
         <v>49</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>27</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>32</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>11</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>45</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>42</v>
       </c>
-      <c r="S7">
-        <v>4</v>
-      </c>
       <c r="T7">
         <v>4</v>
       </c>
       <c r="U7">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="V7">
+        <v>56</v>
+      </c>
+      <c r="W7">
         <v>26</v>
       </c>
-      <c r="W7">
+      <c r="X7">
         <v>55</v>
-      </c>
-      <c r="X7">
-        <v>5</v>
       </c>
       <c r="Y7">
         <v>5</v>
       </c>
       <c r="Z7">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="AA7">
-        <v>65</v>
+        <v>61</v>
+      </c>
+      <c r="AB7">
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -1041,49 +1064,52 @@
         <v>45</v>
       </c>
       <c r="M8">
+        <v>50</v>
+      </c>
+      <c r="N8">
         <v>60</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>40</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>42</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>21</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>59</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>54</v>
-      </c>
-      <c r="S8">
-        <v>14</v>
       </c>
       <c r="T8">
         <v>14</v>
       </c>
       <c r="U8">
+        <v>14</v>
+      </c>
+      <c r="V8">
         <v>65</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <v>36</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>65</v>
       </c>
-      <c r="X8">
-        <v>10</v>
-      </c>
       <c r="Y8">
         <v>10</v>
       </c>
       <c r="Z8">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="AA8">
-        <v>60</v>
+        <v>67</v>
+      </c>
+      <c r="AB8">
+        <v>66</v>
       </c>
     </row>
     <row r="9">
@@ -1135,40 +1161,43 @@
         <v>15</v>
       </c>
       <c r="P9">
+        <v>15</v>
+      </c>
+      <c r="Q9">
         <v>12</v>
       </c>
-      <c r="Q9">
-        <v>15</v>
-      </c>
       <c r="R9">
         <v>15</v>
       </c>
       <c r="S9">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="T9">
         <v>2</v>
       </c>
       <c r="U9">
+        <v>2</v>
+      </c>
+      <c r="V9">
         <v>17</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <v>14</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>17</v>
       </c>
-      <c r="X9">
-        <v>4</v>
-      </c>
       <c r="Y9">
         <v>4</v>
       </c>
       <c r="Z9">
+        <v>4</v>
+      </c>
+      <c r="AA9">
         <v>16</v>
       </c>
-      <c r="AA9">
-        <v>17</v>
+      <c r="AB9">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1211,48 +1240,51 @@
         <v>10</v>
       </c>
       <c r="M10">
+        <v>25</v>
+      </c>
+      <c r="N10">
         <v>18</v>
       </c>
-      <c r="N10">
-        <v>15</v>
-      </c>
       <c r="O10">
+        <v>15</v>
+      </c>
+      <c r="P10">
         <v>13</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>11</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>17</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>18</v>
-      </c>
-      <c r="S10">
-        <v>11</v>
       </c>
       <c r="T10">
         <v>11</v>
       </c>
       <c r="U10">
+        <v>11</v>
+      </c>
+      <c r="V10">
         <v>17</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <v>11</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>22</v>
-      </c>
-      <c r="X10">
-        <v>8</v>
       </c>
       <c r="Y10">
         <v>8</v>
       </c>
       <c r="Z10">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="AA10">
+        <v>18</v>
+      </c>
+      <c r="AB10">
         <v>26</v>
       </c>
     </row>

</xml_diff>